<commit_message>
Add test cases document and update Excel file and renamed
</commit_message>
<xml_diff>
--- a/IT23314092_Assignment 1 - Test cases.xlsx
+++ b/IT23314092_Assignment 1 - Test cases.xlsx
@@ -8,22 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arun/Desktop/test_automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50872258-69D8-FA47-8625-A9256F189A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB23E85E-1439-724F-88C9-E2843326ABF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14800" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Test cases" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">' Test cases'!$G$1:$G$1000</definedName>
-  </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="323">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -49,198 +59,207 @@
     <t>S</t>
   </si>
   <si>
+    <t>mata cake kanna oonee</t>
+  </si>
+  <si>
+    <t>මට පාන් කන්න ඕන</t>
+  </si>
+  <si>
+    <t>මට cake කන්න ඕනේ</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>Neg_002</t>
+  </si>
+  <si>
+    <t>aiye mkkd wune?</t>
+  </si>
+  <si>
+    <t>අයියේ මොකක්ද වුණේ?</t>
+  </si>
+  <si>
+    <t>අයියේ මොකක්ද වුනේ?</t>
+  </si>
+  <si>
+    <t>Neg_003</t>
+  </si>
+  <si>
+    <t>kiyana dhe karapan</t>
+  </si>
+  <si>
+    <t>කියන දෙ කරපන්</t>
+  </si>
+  <si>
+    <t>කියන දේ කරපන්</t>
+  </si>
+  <si>
+    <t>Neg_004</t>
+  </si>
+  <si>
+    <t>suba udhasanak wewa.</t>
+  </si>
+  <si>
+    <t>සුබ උදෑසනක් වේවා.</t>
+  </si>
+  <si>
+    <t>සුබ උදසනක් වේවා.</t>
+  </si>
+  <si>
+    <t>Neg_005</t>
+  </si>
+  <si>
+    <t>mata help ekak dhenna.</t>
+  </si>
+  <si>
+    <t>මට උදව්වක් දෙන්න.</t>
+  </si>
+  <si>
+    <t>මට help එකක් දෙන්න.</t>
+  </si>
+  <si>
+    <t>Neg_006</t>
+  </si>
+  <si>
     <t>PASS</t>
   </si>
   <si>
-    <t>Neg_002</t>
-  </si>
-  <si>
-    <t>aiye mkkd wune?</t>
-  </si>
-  <si>
-    <t>අයියේ මොකක්ද වුණේ?</t>
-  </si>
-  <si>
-    <t>අයියේ මොකක්ද වුනේ?</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>Neg_003</t>
-  </si>
-  <si>
-    <t>Neg_004</t>
-  </si>
-  <si>
-    <t>suba udhasanak wewa.</t>
-  </si>
-  <si>
-    <t>සුබ උදෑසනක් වේවා.</t>
-  </si>
-  <si>
-    <t>කොමන්ඩ් ෆෝර්ම්ස්</t>
+    <t>Neg_007</t>
+  </si>
+  <si>
+    <t>"Nimal" koheda inne?</t>
+  </si>
+  <si>
+    <t>"නිමල්" කොහෙද ඉන්නේ?</t>
+  </si>
+  <si>
+    <t>"නිමල්" කොහේද ඉන්නේ?</t>
+  </si>
+  <si>
+    <t>Neg_008</t>
+  </si>
+  <si>
+    <t>mta nidi mthei...</t>
+  </si>
+  <si>
+    <t>මට නිදි මතයි...</t>
+  </si>
+  <si>
+    <t>මට නිදිමතයි...</t>
+  </si>
+  <si>
+    <t>Neg_009</t>
+  </si>
+  <si>
+    <t>Neg_010</t>
+  </si>
+  <si>
+    <t>Neg_011</t>
+  </si>
+  <si>
+    <t>oya cloud eka danna.</t>
+  </si>
+  <si>
+    <t>ඔයා cloud එක දන්නවද?</t>
+  </si>
+  <si>
+    <t>ඔයා cloud එක දාන්න.</t>
+  </si>
+  <si>
+    <t>Neg_012</t>
+  </si>
+  <si>
+    <t>Neg_013</t>
+  </si>
+  <si>
+    <t>mata Doc ekak ewana.</t>
+  </si>
+  <si>
+    <t>මට Doc එකක් එවන්න.</t>
+  </si>
+  <si>
+    <t>මට ඩොක් එකක් එවන.</t>
+  </si>
+  <si>
+    <t>Neg_014</t>
+  </si>
+  <si>
+    <t>api Galle yamu neda?</t>
+  </si>
+  <si>
+    <t>අපි ගාල්ලේ යමු නේද?</t>
+  </si>
+  <si>
+    <t>අපි Galle යමු නේද?</t>
+  </si>
+  <si>
+    <t>Neg_015</t>
+  </si>
+  <si>
+    <t>5kg bara thiyenawadha.</t>
+  </si>
+  <si>
+    <t>5kg බර තියෙනවා.</t>
+  </si>
+  <si>
+    <t>5kg බර තියෙනවද.</t>
+  </si>
+  <si>
+    <t>Neg_016</t>
+  </si>
+  <si>
+    <t>u mara character ekak.</t>
+  </si>
+  <si>
+    <t>ඌ මාර character එකක්.</t>
+  </si>
+  <si>
+    <t>Neg_017</t>
+  </si>
+  <si>
+    <t>@Kamal mthakadha meka?</t>
+  </si>
+  <si>
+    <t>@Kamal මතකද මේක?</t>
+  </si>
+  <si>
+    <t>කෑමලා මතකද මේක?</t>
+  </si>
+  <si>
+    <t>Neg_018</t>
+  </si>
+  <si>
+    <t>bayai wage 😰</t>
+  </si>
+  <si>
+    <t>බයයි වගේ 😰</t>
+  </si>
+  <si>
+    <t>බයයි වගේ</t>
+  </si>
+  <si>
+    <t>Neg_019</t>
+  </si>
+  <si>
+    <t>eka 75% sure dhennam.</t>
+  </si>
+  <si>
+    <t>ඒක 75% sure දෙන්නම්.</t>
+  </si>
+  <si>
+    <t>Neg_020</t>
+  </si>
+  <si>
+    <t>mama March 12 enawa.</t>
+  </si>
+  <si>
+    <t>මම මාර්තු 12 එනවා.</t>
   </si>
   <si>
     <t>UI Error</t>
   </si>
   <si>
-    <t>Neg_005</t>
-  </si>
-  <si>
-    <t>mata help ekak dhenna.</t>
-  </si>
-  <si>
-    <t>මට උදව්වක් දෙන්න.</t>
-  </si>
-  <si>
-    <t>මට help එකක් දෙන්න.</t>
-  </si>
-  <si>
-    <t>Neg_006</t>
-  </si>
-  <si>
-    <t>ඔව් ඔව්, මම දෙන්නම්.</t>
-  </si>
-  <si>
-    <t>Neg_007</t>
-  </si>
-  <si>
-    <t>"Nimal" koheda inne?</t>
-  </si>
-  <si>
-    <t>"නිමල්" කොහෙද ඉන්නේ?</t>
-  </si>
-  <si>
-    <t>Neg_008</t>
-  </si>
-  <si>
-    <t>mta nidi mthei...</t>
-  </si>
-  <si>
-    <t>මට නිදි මතයි...</t>
-  </si>
-  <si>
-    <t>"නිමල්" කොහේද ඉන්නේ?</t>
-  </si>
-  <si>
-    <t>Neg_009</t>
-  </si>
-  <si>
-    <t>me bike eka lassanai.</t>
-  </si>
-  <si>
-    <t>මේ bike එක ලස්සනයි.</t>
-  </si>
-  <si>
-    <t>මට නිදිමතයි...</t>
-  </si>
-  <si>
-    <t>Neg_010</t>
-  </si>
-  <si>
-    <t>eka mara event ekak.</t>
-  </si>
-  <si>
-    <t>ඒක මාර event එකක්.</t>
-  </si>
-  <si>
-    <t>Neg_011</t>
-  </si>
-  <si>
-    <t>oya cloud eka danna.</t>
-  </si>
-  <si>
-    <t>ඔයා cloud එක දන්නවද?</t>
-  </si>
-  <si>
-    <t>Neg_012</t>
-  </si>
-  <si>
-    <t>mama Instagram damma.</t>
-  </si>
-  <si>
-    <t>මම Instagram දැම්මා.</t>
-  </si>
-  <si>
-    <t>ඔයා cloud එක දාන්න.</t>
-  </si>
-  <si>
-    <t>Neg_013</t>
-  </si>
-  <si>
-    <t>මට Doc එකක් එවන්න.</t>
-  </si>
-  <si>
-    <t>Neg_014</t>
-  </si>
-  <si>
-    <t>api Galle yamu neda?</t>
-  </si>
-  <si>
-    <t>අපි ගාල්ලේ යමු නේද?</t>
-  </si>
-  <si>
-    <t>අපි Galle යමු නේද?</t>
-  </si>
-  <si>
-    <t>Neg_015</t>
-  </si>
-  <si>
-    <t>5kg බර තියෙනවා.</t>
-  </si>
-  <si>
-    <t>Neg_016</t>
-  </si>
-  <si>
-    <t>u mara character ekak.</t>
-  </si>
-  <si>
-    <t>ඌ මාර character එකක්.</t>
-  </si>
-  <si>
-    <t>Neg_017</t>
-  </si>
-  <si>
-    <t>@Kamal mthakadha meka?</t>
-  </si>
-  <si>
-    <t>@Kamal මතකද මේක?</t>
-  </si>
-  <si>
-    <t>කෑමලා මතකද මේක?</t>
-  </si>
-  <si>
-    <t>Neg_018</t>
-  </si>
-  <si>
-    <t>bayai wage 😰</t>
-  </si>
-  <si>
-    <t>බයයි වගේ 😰</t>
-  </si>
-  <si>
-    <t>බයයි වගේ</t>
-  </si>
-  <si>
-    <t>Neg_019</t>
-  </si>
-  <si>
-    <t>eka 75% sure dhennam.</t>
-  </si>
-  <si>
-    <t>ඒක 75% sure දෙන්නම්.</t>
-  </si>
-  <si>
-    <t>Neg_020</t>
-  </si>
-  <si>
-    <t>mama March 12 enawa.</t>
-  </si>
-  <si>
-    <t>මම මාර්තු 12 එනවා.</t>
-  </si>
-  <si>
     <t>Neg_021</t>
   </si>
   <si>
@@ -280,42 +299,45 @@
     <t>විභාග ප්‍රතිඵල එන්න තව දවස් 5ක් තියෙනවා නේද?</t>
   </si>
   <si>
+    <t>ඔයාට party එකට එන්න බැරිද? අපි ගොඩක් fun ගන්න හදන්නේ.</t>
+  </si>
+  <si>
+    <t>Neg_025</t>
+  </si>
+  <si>
+    <t>magea laptop eka repair karanna shop eka close velaa thiyeenne.</t>
+  </si>
+  <si>
+    <t>මගේ ලැප්ටොප් එක රෙපයාර් කරන්න ෂොප් එක ක්ලෝස් වෙලා තියෙන්නේ.</t>
+  </si>
+  <si>
     <t>exam results release වෙන්න තව දවස් 5ක් තියෙනවා නේද?</t>
   </si>
   <si>
-    <t>Neg_025</t>
-  </si>
-  <si>
-    <t>magea laptop eka repair karanna shop eka close velaa thiyeenne.</t>
-  </si>
-  <si>
-    <t>මගේ ලැප්ටොප් එක රෙපයාර් කරන්න ෂොප් එක ක්ලෝස් වෙලා තියෙන්නේ.</t>
+    <t>Neg_026</t>
+  </si>
+  <si>
+    <t>heta 2026/06/15 wenidha kiyala oyaata mathakada?</t>
+  </si>
+  <si>
+    <t>හෙට 2026/06/15 වෙනිදා කියලා ඔයාට මතකද?</t>
   </si>
   <si>
     <t>මගේ laptop එක repair කරන්න shop එක close වෙලා තියෙන්නේ.</t>
   </si>
   <si>
-    <t>Neg_026</t>
-  </si>
-  <si>
-    <t>heta 2026/06/15 wenidha kiyala oyaata mathakada?</t>
-  </si>
-  <si>
-    <t>හෙට 2026/06/15 වෙනිදා කියලා ඔයාට මතකද?</t>
+    <t>Neg_027</t>
+  </si>
+  <si>
+    <t>u mara dial ekak, eya kawadawath wada karanne na.</t>
+  </si>
+  <si>
+    <t>ඌ මාර dial එකක්, එයා කවදාවත් වැඩ කරන්නේ නෑ.</t>
   </si>
   <si>
     <t>හෙට 2026/06/15 වෙනිධ කියලා ඔයාට මතකද?</t>
   </si>
   <si>
-    <t>Neg_027</t>
-  </si>
-  <si>
-    <t>u mara dial ekak, eya kawadawath wada karanne na.</t>
-  </si>
-  <si>
-    <t>ඌ මාර dial එකක්, එයා කවදාවත් වැඩ කරන්නේ නෑ.</t>
-  </si>
-  <si>
     <t>Neg_028</t>
   </si>
   <si>
@@ -343,6 +365,9 @@
     <t>මටනම් පිස්සු වගේ 😵, මේ ඇසයින්මන්ට් එක ගොඩක් අමාරුයි.</t>
   </si>
   <si>
+    <t>මටනම් පිස්සු වගේ, මේ assignment එක ගොඩක් අමාරුයි.</t>
+  </si>
+  <si>
     <t>Neg_031</t>
   </si>
   <si>
@@ -499,9 +524,6 @@
     <t>අද අපි ටීම් එක්ක ෆුල් ප්‍රොජෙක්ට් ස්ටේටස් එක ගැන සාකච්ඡා කරමු, මුලින්ම ගිය සතියේ තියෙන ටාස්ක් ටික හරියට කම්ප්ලීට් වුණාද කියලා චෙක් කරලා, එහෙම වුණත් සමහර ෆයිල්ස් ටික ලේට් වෙන්නේ නිසා ඩොකියුමන්ට්ස් ටික ඇටෑච් කරලා ඊමේල් එකක් මැනේජර්ට යවන්න ඕනේ කියලා අපි කතා කරමු, පස්සේ ටීම්ස් එකේ ලින්ක් එක වට්සැප් කරලා ක්ලයන්ට්ස්ලාට ඩෙමෝ මීටින් එක සෙට් කරන්න පුළුවන් කියලා ප්ලෑන් කරමු. ඔක්කොම තින්ග්ස් සෙට්.</t>
   </si>
   <si>
-    <t>system-on-chip වර්ගයී මේවාඒනි චිපයක් යනු, උපංගය බොධයින් ක්‍රියාත්මකවීමට අවශ්‍ය විවිධ ධාරුදාවන් හෙවත් හද්වේය කොටස් එක්තැන් කොට සැකසූ විශේෂ අර්ධ සන්නායක සැකසුමකි. ඉදිරිඅයීදි නිපදවන ස්මාට් භාවිතයට යෝධ ගාඑනිම පිලිබදව කොළබයින් බැහැර සිටින සියලුම රාජ්ය නිලධරින් දැනුවත් කිරිමට සැළසුම් කර ඇතඑයි ජනඅධිපති කාර්යාලය පවසයි. මේක technology එකේ ලොකු step එකක්.</t>
-  </si>
-  <si>
     <t>Neg_045</t>
   </si>
   <si>
@@ -520,9 +542,6 @@
     <t>CHATGPT අයත් OPENAI සමාගම පසුපස සිටින්නේ වෙන කවුරුවත් නොවී, ලොව ලොකු සල්ලිකාරයෙක් වන එලොන් මස්ක් ය. ලොව ව්‍යවසායකයන් අතර ඉහළින්ම වැජඹෙන ඔහු ටෙස්ලා විදුලි මෝටර් රථ සමාගමේ ද, ප්‍රථම පෞද්ගලික අභ්‍යවකාශ සමාගම වූ ස්පේස් එක්ස් ආයතනයේ ද ආරම්භකයාය. ඔහු මෑතදී ට්විටර් සමාගම ද මිල දී ගත්තේය. එය ලොකු සල්ලිකාරයෙක් නේද?</t>
   </si>
   <si>
-    <t>CHATGPT අයත් OPENAI සමගම පසුපස සිටිනී වෙන කවුරුවත් නොවී, ලොව ලොකු සල්ලි කාරයෙක් වන එලෝන් මුස්ක්‍ය. ලොව ව්යවසායකයන් අතර ඉහළින්ම වැඹෙන ඔහු ටෙස්ලා විදුලි මෝටර්‍රෑත සමගාමී ද, ප්‍රථම පෞද්ගලික අභ්යාවකාශ සමාගම වූ ස්පීස් එක්ස් ආයතනයේ ද අාරම්භකය. ඔහු මාඇතධී ට්විටර් සමාගම ද මිල දී ගත්තේය. එයා ලොකු සල්ලි කාරයෙක් නේද?</t>
-  </si>
-  <si>
     <t>Neg_047</t>
   </si>
   <si>
@@ -532,9 +551,6 @@
     <t>වීකෙන්ඩ් එක එනකොට මම රෙස්ට් කරන්න ප්ලෑන් කළා. අද දවස් වල වැඩ ගොඩක් කරපු නිසා ටයර්ඩ් එකක් තිබ්බා. උදෑසනම ටිකක් නිදාගත්තා පස්සේ බ්‍රෙක්ෆස්ට් එක අරන් රිලැක්ස් වුණා. පස්සේ මූවි එකක් බලලා ටයිම් එක ස්පෙන්ඩ් කළා. දවස් එක ඉවර වෙනකොට නෙක්ස්ට් වීක් එකට රෙඩි වෙන්න පොඩි එනර්ජි එකක් ලැබුණා. ඒත් හෝම්වර්ක් ටික තාම කළේ නෑ. ඔයා මොකක්ද කරන්නේ කියලා කියන්න.</t>
   </si>
   <si>
-    <t>weekend එක එනකොට මම rest කරන්න plan කළා. අද දවස් වල වඩා ගොඩක් කරපු නිසා tired එකක් තිබ්බා. උදෑසනම ටිකක් නිදාගත්තා පස්සේ breakfast එක අරන් relax වුණා. පස්සේ movie එකක් බලලා time එක spend කළා. දවස් එක ඉවර වෙනකොට next week එකට ready වෙන්න පොඩි energy එකක් ලැබුණා. ඒත් homework ටික තවම කළේ නෑ. ඔයා මොකක්ද කරන්නේ කියලා කියන්න.</t>
-  </si>
-  <si>
     <t>Neg_048</t>
   </si>
   <si>
@@ -544,9 +560,6 @@
     <t>මම ගෙදර ගිහිල්ලා තව කෝල් කරන්නම්. අම්මත් එක්ක ෂොපින් යන්න තියෙනවා නිසා මම ෆෝන් එක සයිඩ් එකෙන් තියනවා. අද දවසේ කාලගුණය හරි ලස්සනයි. අපි බීච් එකට යමු කොහොමද? මගේ ඇසයින්මන්ට් එක සබ්මිට් කරන්න ඩෙඩ්ලයින් එක අද 5pm. උදව් කරන්න! ඔයාට කෑම හදන්න පුළුවන් ද? මම හරි බඩගින්නේ ඉන්නේ රයිස් කරි ටිකක් හදන්න.</t>
   </si>
   <si>
-    <t>මම ගෙදර ගිහිල්ලා තව call කරන්නම්. අම්මත් එක්ක shopping යන්න තියෙනවා නිසා මම phone එක side එකෙන් තියනවා. අද දවසේ weather එක හරි ලස්සනයි. අපි beach එකට යමු කොහොමද? මගේ assignment එක submit කරන්න deadline එක අද 5pm. HELP please! ඔයාට කෑම හදන්න පුළුවන් ද? මම හරි බඩගින්නේ ඉන්නේ rice curry ටිකක් හදන්න.</t>
-  </si>
-  <si>
     <t>Neg_049</t>
   </si>
   <si>
@@ -586,21 +599,9 @@
     <t>Neg_053</t>
   </si>
   <si>
-    <t>CHATGPT ayath OPENAI samaagama pasupasa sitinee vena kavuruvath novee, lova loku salli karayek vana Elon Musk ya. lova vYavasaayakayan athara ihaLinma vaeBaeNa ohu tesla vidhuli mootar raTha samaagamee dha, praThama paudhgalika aBHYavakaasha samaagama vuu spees eks aayathanayee dha aarambhakayaaya. ohu maethadhii tvitar samaagama dha mila dhii gaththeeya. Elon Musk kiyanne loku dial ekak.</t>
-  </si>
-  <si>
-    <t>CHATGPT අයත් OPENAI සමාගම පසුපස සිටින්නේ වෙන කවුරුවත් නොවී, ලොව ලොකු සල්ලිකාරයෙක් වන එලොන් මස්ක් ය. ලොව ව්‍යවසායකයන් අතර ඉහළින්ම වැජඹෙන ඔහු ටෙස්ලා විදුලි මෝටර් රථ සමාගමේ ද, ප්‍රථම පෞද්ගලික අභ්‍යවකාශ සමාගම වූ ස්පේස් එක්ස් ආයතනයේ ද ආරම්භකයාය. ඔහු මෑතදී ට්විටර් සමාගම ද මිල දී ගත්තේය. එලොන් මස්ක් කියන්නේ ලොකු ඩයල් එකක්.</t>
-  </si>
-  <si>
     <t>Neg_054</t>
   </si>
   <si>
-    <t>weekend eka enakota mama rest karanna plan kalaa. adha dawas wala wada godak karapu nisaa tired ekak thibba. udhaeesanama tikak nidagaththa passe breakfast eka aran relax vunaa. passe movie ekak balala time eka spend kalaa. dawas eka iwara wenakota next week ekata ready wenna podi energy ekak labunaa. mama hithanne meka hodai kiyala.</t>
-  </si>
-  <si>
-    <t>වීකෙන්ඩ් එක එනකොට මම රෙස්ට් කරන්න ප්ලෑන් කළා. අද දවස් වල වැඩ ගොඩක් කරපු නිසා ටයර්ඩ් එකක් තිබ්බා. උදෑසනම ටිකක් නිදාගත්තා පස්සේ බ්‍රෙක්ෆස්ට් එක අරන් රිලැක්ස් වුණා. පස්සේ මූවි එකක් බලලා ටයිම් එක ස්පෙන්ඩ් කළා. දවස් එක ඉවර වෙනකොට නෙක්ස්ට් වීක් එකට රෙඩි වෙන්න පොඩි එනර්ජි එකක් ලැබුණා. මම හිතන්නේ මේක හොඳයි කියලා.</t>
-  </si>
-  <si>
     <t>Neg_055</t>
   </si>
   <si>
@@ -649,37 +650,58 @@
     <t>Neg_060</t>
   </si>
   <si>
-    <t>exam results release venna thava dhavas 3k thiyenavaa kiyala api news eken daka gaththa. mama hari nervous meka dakkama. nimal kiwwa eyaatath bayai kiyala. api results balala party ekak dhalath balamu. eth results hoda wenna oone neda? mama March 30 wenakam balan inne meka dhenna. mkkd wenne kiyala balamu.</t>
-  </si>
-  <si>
-    <t>විභාග ප්‍රතිඵල එන්න තව දවස් 3ක් තියෙනවා කියලා අපි නිව්ස් එකෙන් දැක ගත්තා. මම හරි නර්වස් මේක දැක්කම. නිමල් කිව්වා එයාටත් බයයි කියලා. අපි රිසල්ට්ස් බලලා පාටියක් දාලත් බලමු. ඒත් රිසල්ට්ස් හොඳ වෙන්න ඕනේ නේද? මම මාර්තු 30 වෙනකම් බලන් ඉන්නේ මේක දෙන්න. මොකක්ද වෙන්නේ කියලා බලමු.</t>
-  </si>
-  <si>
-    <t>මට පාන් කන්න ඕන</t>
-  </si>
-  <si>
-    <t>මට පාන් කන්න ඕනේ</t>
-  </si>
-  <si>
-    <t>mata cake kanna oonee</t>
-  </si>
-  <si>
-    <t>kiyana dhe karapan</t>
-  </si>
-  <si>
-    <t>කියන දෙ කරපන්</t>
-  </si>
-  <si>
-    <t>කියන දේ කරපන්</t>
-  </si>
-  <si>
-    <t>ow oww, mama dennam.</t>
-  </si>
-  <si>
-    <t>mata Doc ekak ewana.</t>
-  </si>
-  <si>
-    <t>5kg bara thiyenawadha.</t>
+    <t>wedi wediyen labewa</t>
+  </si>
+  <si>
+    <t>වැඩි වැඩියෙන් ලැබේවා.</t>
+  </si>
+  <si>
+    <t>වැඩි වැඩියෙන් ලබේවා</t>
+  </si>
+  <si>
+    <t>eya hemin hemin hemin awilla mata baya hithuna machan.</t>
+  </si>
+  <si>
+    <t>එයා හෙමින් හෙමින් හෙමින් ඇවිල්ලා මට බය හිතුණා මචන්.</t>
+  </si>
+  <si>
+    <t>එයා හෙමින් හෙමින් හෙමින් ඇවිල්ලා මට බය හිතුනා මචං.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exam results release venna thava dhavas 3k thiyenavaa kiyala api news eken daka gaththa. mama hari nervous meka dakkama. nimal kiwwa eyaatath bayai kiyala. api results balala party ekak dhalath balamu. eth results hoda wenna oone neda? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">විභාග ප්‍රතිඵල එන්න තව දවස් 3ක් තියෙනවා කියලා අපි නිව්ස් එකෙන් දැක ගත්තා. මම හරි නර්වස් මේක දැක්කම. නිමල් කිව්වා එයාටත් බයයි කියලා. අපි රිසල්ට්ස් බලලා පාටියක් දාලත් බලමු. ඒත් රිසල්ට්ස් හොඳ වෙන්න ඕනේ නේද? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">weekend eka enakota mama rest karanna plan kalaa. adha dawas wala wada godak karapu nisaa tired ekak thibba. udhaeesanama tikak nidagaththa passe breakfast eka aran relax vunaa. passe movie ekak balala time eka spend kalaa. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">වීකෙන්ඩ් එක එනකොට මම රෙස්ට් කරන්න ප්ලෑන් කළා. අද දවස් වල වැඩ ගොඩක් කරපු නිසා ටයර්ඩ් එකක් තිබ්බා. උදෑසනම ටිකක් නිදාගත්තා පස්සේ බ්‍රෙක්ෆස්ට් එක අරන් රිලැක්ස් වුණා. පස්සේ මූවි එකක් බලලා ටයිම් එක ස්පෙන්ඩ් කළා. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHATGPT ayath OPENAI samaagama pasupasa sitinee vena kavuruvath novee, lova loku salli karayek vana Elon Musk ya. lova vYavasaayakayan athara ihaLinma vaeBaeNa ohu tesla vidhuli mootar raTha samaagamee dha, praThama paudhgalika aBHYavakaasha samaagama vuu spees eks aayathanayee dha aarambhakayaaya. ohu maethadhii tvitar samaagama dha mila dhii gaththeeya. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHATGPT අයත් OPENAI සමාගම පසුපස සිටින්නේ වෙන කවුරුවත් නොවී, ලොව ලොකු සල්ලිකාරයෙක් වන එලොන් මස්ක් ය. ලොව ව්‍යවසායකයන් අතර ඉහළින්ම වැජඹෙන ඔහු ටෙස්ලා විදුලි මෝටර් රථ සමාගමේ ද, ප්‍රථම පෞද්ගලික අභ්‍යවකාශ සමාගම වූ ස්පේස් එක්ස් ආයතනයේ ද ආරම්භකයාය. ඔහු මෑතදී ට්විටර් සමාගම ද මිල දී ගත්තේය. </t>
+  </si>
+  <si>
+    <t>mage iPhone 15 eke battery eka 20% ta bahala thibbe kade la.</t>
+  </si>
+  <si>
+    <t>මගේ iPhone 15 එකේ battery එක 20% ට බැහැලා තිබ්බේ කඩේ ලා.</t>
+  </si>
+  <si>
+    <t>මගේ iPhone 15 ඒකේ battery එක 20% ට බහලා තිබ්බේ කඩේ ල.</t>
+  </si>
+  <si>
+    <t>api set wela Galle road eke la 10:30PM wenakam hitiya machan.</t>
+  </si>
+  <si>
+    <t>අපි සෙට් වෙලා Galle road එකේ ලා 10:30PM වෙනකම් හිටියා මචන්.</t>
+  </si>
+  <si>
+    <t>අපි set වෙලා Galle road එකේ ල 10:30PM වෙනකම් හිටියා මචන්.</t>
   </si>
   <si>
     <t>Singlish input types covered</t>
@@ -688,6 +710,9 @@
     <t>Evidence or rationale for the input type covered</t>
   </si>
   <si>
+    <t>Command forms</t>
+  </si>
+  <si>
     <t>Informal variation of a common question.</t>
   </si>
   <si>
@@ -697,9 +722,6 @@
     <t>Shorthand 'mkkd' for 'mokada'.</t>
   </si>
   <si>
-    <t>Command forms</t>
-  </si>
-  <si>
     <t>Short urgent command with punctuation.</t>
   </si>
   <si>
@@ -733,27 +755,12 @@
     <t>Shorthand with trailing ellipsis.</t>
   </si>
   <si>
-    <t>Isolated English Words</t>
-  </si>
-  <si>
-    <t>Use of 'bike' in a short sentence.</t>
-  </si>
-  <si>
-    <t>Use of 'event' in a short sentence.</t>
-  </si>
-  <si>
     <t>English Digital Terms</t>
   </si>
   <si>
     <t>Use of 'cloud' as a technical term.</t>
   </si>
   <si>
-    <t>Platform Names</t>
-  </si>
-  <si>
-    <t>Social media platform name.</t>
-  </si>
-  <si>
     <t>English Clipped Forms</t>
   </si>
   <si>
@@ -980,6 +987,21 @@
   </si>
   <si>
     <t>Academic results anticipation narrative.</t>
+  </si>
+  <si>
+    <t>emphasis that standard transliterators often misinterpret or fail to convert consistently.</t>
+  </si>
+  <si>
+    <t>Brand Names / Numbers /Slang</t>
+  </si>
+  <si>
+    <t>Contains a brand name ("iPhone 15"), a numerical percentage ("20%"), and the informal location suffix "la" which complicates the tokenization process.</t>
+  </si>
+  <si>
+    <t>Place Names / Time Formats / Slang</t>
+  </si>
+  <si>
+    <t>Combines a specific English place name ("Galle road"), a rigid time format ("10:30PM"), and the casual "la" suffix within a single medium-length sentence</t>
   </si>
 </sst>
 </file>
@@ -1043,7 +1065,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1058,7 +1080,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1353,7 +1379,7 @@
     <col min="10" max="11" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:25" ht="79" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:23" ht="79" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1372,14 +1398,14 @@
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="2" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H1" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1387,22 +1413,22 @@
         <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>212</v>
+        <v>8</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>210</v>
+        <v>9</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>211</v>
+        <v>10</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>221</v>
+        <v>11</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>226</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -1418,33 +1444,31 @@
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
       <c r="W2" s="2"/>
-      <c r="X2" s="2"/>
-      <c r="Y2" s="2"/>
-    </row>
-    <row r="3" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>223</v>
+      <c r="H3" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>228</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
@@ -1460,33 +1484,31 @@
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-    </row>
-    <row r="4" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>213</v>
+        <v>17</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>214</v>
+        <v>18</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>215</v>
+        <v>19</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="I4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>225</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>229</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -1502,33 +1524,31 @@
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
-    </row>
-    <row r="5" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>227</v>
+        <v>11</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>231</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
@@ -1544,33 +1564,31 @@
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
-    </row>
-    <row r="6" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>229</v>
+        <v>11</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>233</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -1586,73 +1604,71 @@
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
-    </row>
-    <row r="7" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="3" t="s">
+    </row>
+    <row r="7" spans="2:23" s="8" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>13</v>
+      <c r="D7" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2"/>
-      <c r="Y7" s="2"/>
-    </row>
-    <row r="8" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+    </row>
+    <row r="8" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="G8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>233</v>
+        <v>11</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>237</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
@@ -1668,33 +1684,31 @@
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
-    </row>
-    <row r="9" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>235</v>
+        <v>11</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>239</v>
       </c>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
@@ -1710,94 +1724,88 @@
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
-      <c r="X9" s="2"/>
-      <c r="Y9" s="2"/>
-    </row>
-    <row r="10" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>13</v>
+    </row>
+    <row r="10" spans="2:23" s="8" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
-      <c r="Y10" s="2"/>
-    </row>
-    <row r="11" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="7"/>
+      <c r="T10" s="7"/>
+      <c r="U10" s="7"/>
+      <c r="V10" s="7"/>
+      <c r="W10" s="7"/>
+    </row>
+    <row r="11" spans="2:23" s="8" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>13</v>
+      <c r="C11" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>236</v>
+        <v>319</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
-      <c r="Y11" s="2"/>
-    </row>
-    <row r="12" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+        <v>320</v>
+      </c>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="7"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="7"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="7"/>
+    </row>
+    <row r="12" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
         <v>40</v>
       </c>
@@ -1811,16 +1819,16 @@
         <v>42</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="I12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>240</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>241</v>
       </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
@@ -1836,75 +1844,71 @@
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
-      <c r="X12" s="2"/>
-      <c r="Y12" s="2"/>
-    </row>
-    <row r="13" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="3" t="s">
+    </row>
+    <row r="13" spans="2:23" s="8" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="C13" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
+      <c r="R13" s="7"/>
+      <c r="S13" s="7"/>
+      <c r="T13" s="7"/>
+      <c r="U13" s="7"/>
+      <c r="V13" s="7"/>
+      <c r="W13" s="7"/>
+    </row>
+    <row r="14" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
-      <c r="Y13" s="2"/>
-    </row>
-    <row r="14" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="3" t="s">
-        <v>47</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>217</v>
+        <v>46</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>48</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>244</v>
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -1920,10 +1924,8 @@
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
-      <c r="Y14" s="2"/>
-    </row>
-    <row r="15" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
         <v>49</v>
       </c>
@@ -1940,13 +1942,13 @@
         <v>52</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="I15" s="3" t="s">
         <v>245</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>246</v>
       </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
@@ -1962,10 +1964,8 @@
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
-      <c r="Y15" s="2"/>
-    </row>
-    <row r="16" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3" t="s">
         <v>53</v>
       </c>
@@ -1973,22 +1973,22 @@
         <v>7</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>218</v>
+        <v>54</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H16" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>248</v>
       </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
@@ -2004,33 +2004,31 @@
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
       <c r="W16" s="2"/>
-      <c r="X16" s="2"/>
-      <c r="Y16" s="2"/>
-    </row>
-    <row r="17" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="I17" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>250</v>
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
@@ -2046,33 +2044,31 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
-      <c r="X17" s="2"/>
-      <c r="Y17" s="2"/>
-    </row>
-    <row r="18" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>251</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>252</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -2088,33 +2084,31 @@
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
       <c r="W18" s="2"/>
-      <c r="X18" s="2"/>
-      <c r="Y18" s="2"/>
-    </row>
-    <row r="19" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="I19" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>254</v>
       </c>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -2130,31 +2124,31 @@
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2"/>
-      <c r="X19" s="2"/>
-      <c r="Y19" s="2"/>
-    </row>
-    <row r="20" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F20" s="3"/>
+        <v>70</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>70</v>
+      </c>
       <c r="G20" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H20" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>255</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>256</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -2170,33 +2164,31 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="W20" s="2"/>
-      <c r="X20" s="2"/>
-      <c r="Y20" s="2"/>
-    </row>
-    <row r="21" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="G21" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H21" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="I21" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>258</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
@@ -2212,33 +2204,31 @@
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
       <c r="W21" s="2"/>
-      <c r="X21" s="2"/>
-      <c r="Y21" s="2"/>
-    </row>
-    <row r="22" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="G22" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H22" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="I22" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>260</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -2254,33 +2244,31 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
-      <c r="X22" s="2"/>
-      <c r="Y22" s="2"/>
-    </row>
-    <row r="23" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="D23" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E23" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F23" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="G23" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="I23" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>262</v>
       </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
@@ -2296,33 +2284,31 @@
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
       <c r="W23" s="2"/>
-      <c r="X23" s="2"/>
-      <c r="Y23" s="2"/>
-    </row>
-    <row r="24" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E24" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F24" s="3" t="s">
-        <v>78</v>
-      </c>
       <c r="G24" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>263</v>
+        <v>11</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>262</v>
       </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -2338,33 +2324,31 @@
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
       <c r="W24" s="2"/>
-      <c r="X24" s="2"/>
-      <c r="Y24" s="2"/>
-    </row>
-    <row r="25" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>264</v>
+        <v>11</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>263</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -2380,33 +2364,31 @@
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
       <c r="W25" s="2"/>
-      <c r="X25" s="2"/>
-      <c r="Y25" s="2"/>
-    </row>
-    <row r="26" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>265</v>
+        <v>11</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>264</v>
       </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
@@ -2422,33 +2404,31 @@
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
       <c r="W26" s="2"/>
-      <c r="X26" s="2"/>
-      <c r="Y26" s="2"/>
-    </row>
-    <row r="27" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>266</v>
+        <v>11</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>265</v>
       </c>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -2464,33 +2444,31 @@
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
       <c r="W27" s="2"/>
-      <c r="X27" s="2"/>
-      <c r="Y27" s="2"/>
-    </row>
-    <row r="28" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="I28" s="6" t="s">
-        <v>267</v>
+        <v>11</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>266</v>
       </c>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -2506,31 +2484,31 @@
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2"/>
-      <c r="X28" s="2"/>
-      <c r="Y28" s="2"/>
-    </row>
-    <row r="29" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F29" s="3"/>
+        <v>103</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>103</v>
+      </c>
       <c r="G29" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H29" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>268</v>
+        <v>29</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>267</v>
       </c>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
@@ -2546,33 +2524,31 @@
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
-      <c r="X29" s="2"/>
-      <c r="Y29" s="2"/>
-    </row>
-    <row r="30" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="I30" s="6" t="s">
-        <v>269</v>
+        <v>29</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>268</v>
       </c>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
@@ -2588,31 +2564,31 @@
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
       <c r="W30" s="2"/>
-      <c r="X30" s="2"/>
-      <c r="Y30" s="2"/>
-    </row>
-    <row r="31" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F31" s="3"/>
+        <v>109</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="G31" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>270</v>
+        <v>11</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>269</v>
       </c>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
@@ -2628,33 +2604,31 @@
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
       <c r="W31" s="2"/>
-      <c r="X31" s="2"/>
-      <c r="Y31" s="2"/>
-    </row>
-    <row r="32" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>271</v>
+        <v>11</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>270</v>
       </c>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
@@ -2670,33 +2644,31 @@
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
       <c r="W32" s="2"/>
-      <c r="X32" s="2"/>
-      <c r="Y32" s="2"/>
-    </row>
-    <row r="33" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="I33" s="6" t="s">
-        <v>272</v>
+        <v>74</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>271</v>
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
@@ -2712,33 +2684,31 @@
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
       <c r="W33" s="2"/>
-      <c r="X33" s="2"/>
-      <c r="Y33" s="2"/>
-    </row>
-    <row r="34" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="I34" s="6" t="s">
-        <v>273</v>
+        <v>11</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>272</v>
       </c>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
@@ -2754,33 +2724,31 @@
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
       <c r="W34" s="2"/>
-      <c r="X34" s="2"/>
-      <c r="Y34" s="2"/>
-    </row>
-    <row r="35" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="I35" s="6" t="s">
-        <v>274</v>
+        <v>11</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>273</v>
       </c>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
@@ -2796,33 +2764,31 @@
       <c r="U35" s="2"/>
       <c r="V35" s="2"/>
       <c r="W35" s="2"/>
-      <c r="X35" s="2"/>
-      <c r="Y35" s="2"/>
-    </row>
-    <row r="36" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="3" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H36" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="I36" s="3" t="s">
         <v>275</v>
-      </c>
-      <c r="I36" s="6" t="s">
-        <v>276</v>
       </c>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
@@ -2838,33 +2804,31 @@
       <c r="U36" s="2"/>
       <c r="V36" s="2"/>
       <c r="W36" s="2"/>
-      <c r="X36" s="2"/>
-      <c r="Y36" s="2"/>
-    </row>
-    <row r="37" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="3" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H37" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="I37" s="6" t="s">
-        <v>277</v>
+        <v>29</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>276</v>
       </c>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
@@ -2880,33 +2844,31 @@
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
       <c r="W37" s="2"/>
-      <c r="X37" s="2"/>
-      <c r="Y37" s="2"/>
-    </row>
-    <row r="38" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="3" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H38" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="I38" s="3" t="s">
         <v>278</v>
-      </c>
-      <c r="I38" s="6" t="s">
-        <v>279</v>
       </c>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
@@ -2922,33 +2884,31 @@
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
       <c r="W38" s="2"/>
-      <c r="X38" s="2"/>
-      <c r="Y38" s="2"/>
-    </row>
-    <row r="39" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H39" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="I39" s="3" t="s">
         <v>280</v>
-      </c>
-      <c r="I39" s="6" t="s">
-        <v>281</v>
       </c>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
@@ -2964,33 +2924,31 @@
       <c r="U39" s="2"/>
       <c r="V39" s="2"/>
       <c r="W39" s="2"/>
-      <c r="X39" s="2"/>
-      <c r="Y39" s="2"/>
-    </row>
-    <row r="40" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="I40" s="6" t="s">
-        <v>282</v>
+        <v>11</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>281</v>
       </c>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
@@ -3006,33 +2964,31 @@
       <c r="U40" s="2"/>
       <c r="V40" s="2"/>
       <c r="W40" s="2"/>
-      <c r="X40" s="2"/>
-      <c r="Y40" s="2"/>
-    </row>
-    <row r="41" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H41" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="I41" s="6" t="s">
-        <v>283</v>
+        <v>29</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>282</v>
       </c>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
@@ -3048,33 +3004,31 @@
       <c r="U41" s="2"/>
       <c r="V41" s="2"/>
       <c r="W41" s="2"/>
-      <c r="X41" s="2"/>
-      <c r="Y41" s="2"/>
-    </row>
-    <row r="42" spans="2:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="2:23" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H42" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="I42" s="3" t="s">
         <v>284</v>
-      </c>
-      <c r="I42" s="6" t="s">
-        <v>285</v>
       </c>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
@@ -3090,33 +3044,31 @@
       <c r="U42" s="2"/>
       <c r="V42" s="2"/>
       <c r="W42" s="2"/>
-      <c r="X42" s="2"/>
-      <c r="Y42" s="2"/>
-    </row>
-    <row r="43" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="3" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H43" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="I43" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="I43" s="6" t="s">
-        <v>287</v>
       </c>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
@@ -3132,31 +3084,29 @@
       <c r="U43" s="2"/>
       <c r="V43" s="2"/>
       <c r="W43" s="2"/>
-      <c r="X43" s="2"/>
-      <c r="Y43" s="2"/>
-    </row>
-    <row r="44" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="3" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="I44" s="6" t="s">
-        <v>288</v>
+        <v>11</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>287</v>
       </c>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
@@ -3172,33 +3122,29 @@
       <c r="U44" s="2"/>
       <c r="V44" s="2"/>
       <c r="W44" s="2"/>
-      <c r="X44" s="2"/>
-      <c r="Y44" s="2"/>
-    </row>
-    <row r="45" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="3" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>158</v>
-      </c>
+        <v>162</v>
+      </c>
+      <c r="F45" s="3"/>
       <c r="G45" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H45" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="I45" s="3" t="s">
         <v>289</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>290</v>
       </c>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
@@ -3214,31 +3160,29 @@
       <c r="U45" s="2"/>
       <c r="V45" s="2"/>
       <c r="W45" s="2"/>
-      <c r="X45" s="2"/>
-      <c r="Y45" s="2"/>
-    </row>
-    <row r="46" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="3" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H46" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="I46" s="3" t="s">
         <v>291</v>
-      </c>
-      <c r="I46" s="6" t="s">
-        <v>292</v>
       </c>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
@@ -3254,33 +3198,29 @@
       <c r="U46" s="2"/>
       <c r="V46" s="2"/>
       <c r="W46" s="2"/>
-      <c r="X46" s="2"/>
-      <c r="Y46" s="2"/>
-    </row>
-    <row r="47" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="3" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>165</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="F47" s="3"/>
       <c r="G47" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H47" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="I47" s="3" t="s">
         <v>293</v>
-      </c>
-      <c r="I47" s="6" t="s">
-        <v>294</v>
       </c>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
@@ -3296,33 +3236,29 @@
       <c r="U47" s="2"/>
       <c r="V47" s="2"/>
       <c r="W47" s="2"/>
-      <c r="X47" s="2"/>
-      <c r="Y47" s="2"/>
-    </row>
-    <row r="48" spans="2:25" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="2:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F48" s="3" t="s">
-        <v>169</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="F48" s="3"/>
       <c r="G48" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H48" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="I48" s="3" t="s">
         <v>295</v>
-      </c>
-      <c r="I48" s="6" t="s">
-        <v>296</v>
       </c>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
@@ -3338,33 +3274,29 @@
       <c r="U48" s="2"/>
       <c r="V48" s="2"/>
       <c r="W48" s="2"/>
-      <c r="X48" s="2"/>
-      <c r="Y48" s="2"/>
     </row>
     <row r="49" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>173</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="F49" s="3"/>
       <c r="G49" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H49" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="I49" s="3" t="s">
         <v>297</v>
-      </c>
-      <c r="I49" s="6" t="s">
-        <v>298</v>
       </c>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
@@ -3380,31 +3312,29 @@
       <c r="U49" s="2"/>
       <c r="V49" s="2"/>
       <c r="W49" s="2"/>
-      <c r="X49" s="2"/>
-      <c r="Y49" s="2"/>
     </row>
     <row r="50" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H50" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="I50" s="3" t="s">
         <v>299</v>
-      </c>
-      <c r="I50" s="6" t="s">
-        <v>300</v>
       </c>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
@@ -3420,31 +3350,29 @@
       <c r="U50" s="2"/>
       <c r="V50" s="2"/>
       <c r="W50" s="2"/>
-      <c r="X50" s="2"/>
-      <c r="Y50" s="2"/>
     </row>
     <row r="51" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H51" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="I51" s="6" t="s">
-        <v>301</v>
+        <v>11</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>300</v>
       </c>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
@@ -3460,31 +3388,29 @@
       <c r="U51" s="2"/>
       <c r="V51" s="2"/>
       <c r="W51" s="2"/>
-      <c r="X51" s="2"/>
-      <c r="Y51" s="2"/>
     </row>
     <row r="52" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="I52" s="6" t="s">
-        <v>302</v>
+        <v>11</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>301</v>
       </c>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
@@ -3500,31 +3426,29 @@
       <c r="U52" s="2"/>
       <c r="V52" s="2"/>
       <c r="W52" s="2"/>
-      <c r="X52" s="2"/>
-      <c r="Y52" s="2"/>
     </row>
     <row r="53" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H53" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="I53" s="6" t="s">
-        <v>303</v>
+        <v>11</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>302</v>
       </c>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
@@ -3540,31 +3464,29 @@
       <c r="U53" s="2"/>
       <c r="V53" s="2"/>
       <c r="W53" s="2"/>
-      <c r="X53" s="2"/>
-      <c r="Y53" s="2"/>
     </row>
     <row r="54" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>187</v>
+        <v>215</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H54" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="I54" s="3" t="s">
         <v>304</v>
-      </c>
-      <c r="I54" s="6" t="s">
-        <v>305</v>
       </c>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
@@ -3580,31 +3502,29 @@
       <c r="U54" s="2"/>
       <c r="V54" s="2"/>
       <c r="W54" s="2"/>
-      <c r="X54" s="2"/>
-      <c r="Y54" s="2"/>
     </row>
     <row r="55" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H55" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="I55" s="6" t="s">
-        <v>306</v>
+        <v>11</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>305</v>
       </c>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
@@ -3620,31 +3540,29 @@
       <c r="U55" s="2"/>
       <c r="V55" s="2"/>
       <c r="W55" s="2"/>
-      <c r="X55" s="2"/>
-      <c r="Y55" s="2"/>
     </row>
     <row r="56" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="3" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H56" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="I56" s="3" t="s">
         <v>307</v>
-      </c>
-      <c r="I56" s="6" t="s">
-        <v>308</v>
       </c>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
@@ -3660,31 +3578,29 @@
       <c r="U56" s="2"/>
       <c r="V56" s="2"/>
       <c r="W56" s="2"/>
-      <c r="X56" s="2"/>
-      <c r="Y56" s="2"/>
     </row>
     <row r="57" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H57" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="I57" s="3" t="s">
         <v>309</v>
-      </c>
-      <c r="I57" s="6" t="s">
-        <v>310</v>
       </c>
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
@@ -3700,31 +3616,29 @@
       <c r="U57" s="2"/>
       <c r="V57" s="2"/>
       <c r="W57" s="2"/>
-      <c r="X57" s="2"/>
-      <c r="Y57" s="2"/>
     </row>
     <row r="58" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="3" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H58" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="I58" s="3" t="s">
         <v>311</v>
-      </c>
-      <c r="I58" s="6" t="s">
-        <v>312</v>
       </c>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
@@ -3740,31 +3654,29 @@
       <c r="U58" s="2"/>
       <c r="V58" s="2"/>
       <c r="W58" s="2"/>
-      <c r="X58" s="2"/>
-      <c r="Y58" s="2"/>
     </row>
     <row r="59" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="3" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H59" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="I59" s="3" t="s">
         <v>313</v>
-      </c>
-      <c r="I59" s="6" t="s">
-        <v>314</v>
       </c>
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
@@ -3780,31 +3692,29 @@
       <c r="U59" s="2"/>
       <c r="V59" s="2"/>
       <c r="W59" s="2"/>
-      <c r="X59" s="2"/>
-      <c r="Y59" s="2"/>
     </row>
     <row r="60" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="3" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H60" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="I60" s="3" t="s">
         <v>315</v>
-      </c>
-      <c r="I60" s="6" t="s">
-        <v>316</v>
       </c>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
@@ -3820,31 +3730,29 @@
       <c r="U60" s="2"/>
       <c r="V60" s="2"/>
       <c r="W60" s="2"/>
-      <c r="X60" s="2"/>
-      <c r="Y60" s="2"/>
     </row>
     <row r="61" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="3" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H61" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="I61" s="3" t="s">
         <v>317</v>
-      </c>
-      <c r="I61" s="6" t="s">
-        <v>318</v>
       </c>
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
@@ -3860,8 +3768,6 @@
       <c r="U61" s="2"/>
       <c r="V61" s="2"/>
       <c r="W61" s="2"/>
-      <c r="X61" s="2"/>
-      <c r="Y61" s="2"/>
     </row>
     <row r="62" spans="2:27" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="4"/>

</xml_diff>